<commit_message>
Rename Plates pendant Farsi heading from آویز پلیتس to پلیتس
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/محصولات_آذران_نور.xlsx
+++ b/محصولات_آذران_نور.xlsx
@@ -1312,7 +1312,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>آویز پلیتس</t>
+          <t>پلیتس</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -9559,7 +9559,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>آویز پلیتس</t>
+          <t>پلیتس</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -9584,7 +9584,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>آویز پلیتس</t>
+          <t>پلیتس</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -9609,7 +9609,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>آویز پلیتس</t>
+          <t>پلیتس</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">

</xml_diff>